<commit_message>
Update excel_to_json.py to extract txt and update readme
</commit_message>
<xml_diff>
--- a/monitor_xlsx/20260119.xlsx
+++ b/monitor_xlsx/20260119.xlsx
@@ -544,10 +544,6 @@
           <t>+1.68%</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -570,10 +566,6 @@
           <t>-0.60%</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -596,10 +588,6 @@
           <t>+0.15%</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -622,10 +610,6 @@
           <t>+1.15%</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -648,10 +632,6 @@
           <t>+0.13%</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -669,7 +649,6 @@
           <t>-277.95億</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>81.87億</t>
@@ -707,7 +686,6 @@
           <t>-131.23億</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>-73.81億</t>
@@ -718,8 +696,6 @@
           <t>-369.06億</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -737,15 +713,11 @@
           <t>128.98%</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>None%</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -763,11 +735,6 @@
           <t>-462.18億</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -785,15 +752,11 @@
           <t>13182口</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>13159口</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -811,7 +774,6 @@
           <t>-63.23億</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>-30.03億</t>
@@ -916,10 +878,6 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-    </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1041,7 +999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W20"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1076,6 +1034,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -1267,7 +1226,6 @@
           <t>S&amp;P黃金正2</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="G5" s="6" t="n">
         <v>-114</v>
       </c>
@@ -2127,46 +2085,46 @@
           <t>智邦</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>上市</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
+      <c r="C19" t="n">
         <v>1165</v>
       </c>
+      <c r="D19" s="7" t="n">
+        <v>-5.28</v>
+      </c>
       <c r="E19" s="7" t="n">
-        <v>-5.28</v>
-      </c>
-      <c r="F19" t="n">
         <v>4631</v>
       </c>
+      <c r="F19" s="6" t="n">
+        <v>-160</v>
+      </c>
       <c r="G19" s="6" t="n">
-        <v>-160</v>
+        <v>198</v>
       </c>
       <c r="H19" t="n">
-        <v>36</v>
+        <v>-514</v>
       </c>
       <c r="I19" t="n">
-        <v>-514</v>
+        <v>-293</v>
       </c>
       <c r="J19" t="n">
-        <v>64</v>
+        <v>251</v>
       </c>
       <c r="K19" t="n">
-        <v>251</v>
+        <v>2643</v>
       </c>
       <c r="L19" t="n">
-        <v>2643</v>
+        <v>13885</v>
       </c>
       <c r="M19" t="n">
-        <v>14071</v>
+        <v>-140153</v>
       </c>
       <c r="N19" t="n">
-        <v>-140153</v>
-      </c>
-      <c r="O19" t="n">
-        <v>-4.04</v>
+        <v>-3.39</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>中性</t>
+        </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
@@ -2239,6 +2197,59 @@
       <c r="W20" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2404</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>漢唐</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1095</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3112</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>-211</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1268</v>
+      </c>
+      <c r="H21" t="n">
+        <v>489</v>
+      </c>
+      <c r="I21" t="n">
+        <v>269</v>
+      </c>
+      <c r="J21" t="n">
+        <v>168</v>
+      </c>
+      <c r="K21" t="n">
+        <v>2239</v>
+      </c>
+      <c r="L21" t="n">
+        <v>11598</v>
+      </c>
+      <c r="M21" t="n">
+        <v>-47585</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>偏多</t>
         </is>
       </c>
     </row>

</xml_diff>